<commit_message>
Updated THA_grids_kan model - 2026-05-06 23:09
</commit_message>
<xml_diff>
--- a/VerveStacks_THA_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_THA_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_THA_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E9656238-3385-42BA-BF96-15E0EC23A838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{423F7971-FB0F-43FF-BE9E-236134DB7701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4657,7 +4657,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7962B592-61F7-444C-BDB5-69C3C3CCCB02}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C268C30E-98A5-4DC8-BD37-C718B4FEFCC8}">
   <dimension ref="B9:H288"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -29119,7 +29119,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A31BADFB-CA5D-465A-9632-7E83DBE6EE2C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F5F00FD-6C0D-4581-A9FF-7A22DB117714}">
   <dimension ref="B9:L288"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>